<commit_message>
Refactor README and scripts for improved clarity and functionality
</commit_message>
<xml_diff>
--- a/step2_alignment/report/clik_as_is_results.xlsx
+++ b/step2_alignment/report/clik_as_is_results.xlsx
@@ -442,7 +442,7 @@
   <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="52" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="30" customWidth="1" min="4" max="4"/>
@@ -539,7 +539,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Mediane e tasso di vittoria</t>
+          <t>Mediane per caso</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -554,7 +554,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>CLIK migliore su</t>
+          <t>CLIK migliore in</t>
         </is>
       </c>
     </row>
@@ -565,14 +565,14 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>8.99</v>
+        <v>9.279999999999999</v>
       </c>
       <c r="C7" t="n">
-        <v>8.59</v>
+        <v>9.49</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>48% dei denti</t>
+          <t>44% dei casi</t>
         </is>
       </c>
     </row>
@@ -583,14 +583,14 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1.81</v>
+        <v>1.84</v>
       </c>
       <c r="C8" t="n">
-        <v>1.58</v>
+        <v>1.76</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>43% dei denti</t>
+          <t>33% dei casi</t>
         </is>
       </c>
     </row>
@@ -601,21 +601,21 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>2.47</v>
+        <v>2.56</v>
       </c>
       <c r="C9" t="n">
-        <v>1.53</v>
+        <v>1.72</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>24% dei denti</t>
+          <t>17% dei casi</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Soggetti valutati</t>
+          <t>Casi valutati</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -635,7 +635,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Denti esclusi - estratti durante il trattamento</t>
+          <t>Denti esclusi - assenti dal piano simulato</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -645,7 +645,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Denti esclusi - rimeshati tra i due stadi</t>
+          <t>Denti esclusi - numero di vertici diverso tra i due stadi</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -2302,7 +2302,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.0034</v>
+        <v>0.0033</v>
       </c>
       <c r="C2" t="n">
         <v>0.24</v>
@@ -2318,10 +2318,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.3831</v>
+        <v>0.3972</v>
       </c>
       <c r="C3" t="n">
-        <v>4.3</v>
+        <v>4.26</v>
       </c>
       <c r="D3" t="n">
         <v>40</v>
@@ -2334,10 +2334,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.1541</v>
+        <v>0.1407</v>
       </c>
       <c r="C4" t="n">
-        <v>0.98</v>
+        <v>1</v>
       </c>
       <c r="D4" t="n">
         <v>40</v>
@@ -2423,7 +2423,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2.12e-02</t>
+          <t>2.13e-02</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -2603,7 +2603,7 @@
         <v>1576</v>
       </c>
       <c r="C4" t="n">
-        <v>9.186</v>
+        <v>9.185</v>
       </c>
       <c r="D4" t="n">
         <v>8.91</v>
@@ -2658,9 +2658,9 @@
   <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="78" customWidth="1" min="3" max="3"/>
+    <col width="90" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2698,22 +2698,22 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Estratti durante il trattamento</t>
+          <t>Assenti dal piano simulato</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>335</v>
+        <v>232</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>assenti nel post; CLIK non lo sa e li sposta comunque di 2.68 mm mediani</t>
+          <t>oltre ai 78 terzi molari assenti; i dati non dicono se siano stati estratti, e CLIK li sposta comunque di 1.72 mm mediani</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Rimeshati fra i due stadi</t>
+          <t>Numero di vertici diverso fra i due stadi</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -2848,7 +2848,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>La diffusion e' generativa, quindi ogni esecuzione campiona diversamente. Il divario dal baseline e' circa 11 volte la dispersione fra seed: l'errore misurato e' sistematico e non rumore, e valutare con un solo seed era affidabile.</t>
+          <t>La diffusion e' generativa, quindi ogni esecuzione campiona diversamente. Il divario dal baseline e' circa quindici volte la dispersione fra seed: l'errore misurato e' sistematico e non rumore, e valutare con un solo seed era affidabile.</t>
         </is>
       </c>
     </row>

</xml_diff>